<commit_message>
Trabajo pendiente: armonización, Mincer y Gini
Cambios que ya estaban en el árbol de trabajo, sin relación con la
extensión de empleo_pleno_rama.do:

- empleo_adecuado_serie.do: documentación de la adaptación multi-año
  (renombres p##, códigos de p21/p25/p27/p28/p32/p34 por período).
- armonizacion_empleo adecuado.do: rutas portables, corrección del
  rename del CSV de salarios y bloque urbano/nacional; se advierte en
  el encabezado que el ingreso y las horas de los 90 no se limpian bien
  y que la versión correcta es la del paper de Íconos.
- educ_ingrl_hora.do / _fig.do: controles por rama de actividad en la
  regresión y notas al pie acordes.
- gini_decomp5.do: se quita la definición local de $gd y $gh_root; la
  raíz la fija el master.
- gini_decomposition.xlsx: salida regenerada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
+++ b/Dashboards/data/Data final/desigualdad/gini_decomposition.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="17" uniqueCount="17">
   <si>
     <t>slaboral</t>
   </si>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -244,10 +244,10 @@
         <v>0.75429217680282479</v>
       </c>
       <c r="I3" s="1">
-        <v>0.95194766651444362</v>
+        <v>0.95194766651444363</v>
       </c>
       <c r="J3" s="1">
-        <v>0.73375117507014342</v>
+        <v>0.73375117507014343</v>
       </c>
       <c r="K3" s="1">
         <v>0.66097397909885669</v>
@@ -477,7 +477,7 @@
         <v>-0.0001102270867625</v>
       </c>
       <c r="P7" s="1">
-        <v>-0.031185044427598198</v>
+        <v>-0.031185044427598199</v>
       </c>
       <c r="Q7" s="1">
         <v>2011</v>
@@ -500,7 +500,7 @@
         <v>0.53141866575384633</v>
       </c>
       <c r="F8" s="1">
-        <v>0.91971154305627389</v>
+        <v>0.9197115430562739</v>
       </c>
       <c r="G8" s="1">
         <v>0.98401130653132307</v>
@@ -509,7 +509,7 @@
         <v>0.77463588021538399</v>
       </c>
       <c r="I8" s="1">
-        <v>0.9363005277007389</v>
+        <v>0.93630052770073891</v>
       </c>
       <c r="J8" s="1">
         <v>0.64337824094114437</v>
@@ -618,7 +618,7 @@
         <v>0.92538183041701216</v>
       </c>
       <c r="J10" s="1">
-        <v>0.57802712932923916</v>
+        <v>0.57802712932923917</v>
       </c>
       <c r="K10" s="1">
         <v>0.49262858230414758</v>
@@ -680,7 +680,7 @@
         <v>-0.3121255338443033</v>
       </c>
       <c r="M11" s="1">
-        <v>0.00049913281635660005</v>
+        <v>0.00049913281635660006</v>
       </c>
       <c r="N11" s="1">
         <v>0.025702756408549399</v>
@@ -730,7 +730,7 @@
         <v>0.41536560745237261</v>
       </c>
       <c r="L12" s="1">
-        <v>-0.32294752797140241</v>
+        <v>-0.32294752797140242</v>
       </c>
       <c r="M12" s="1">
         <v>0.029985990470625199</v>
@@ -777,7 +777,7 @@
         <v>0.90866866567465843</v>
       </c>
       <c r="J13" s="1">
-        <v>0.59074717444760227</v>
+        <v>0.59074717444760228</v>
       </c>
       <c r="K13" s="1">
         <v>0.48290553645140061</v>

</xml_diff>